<commit_message>
Fix data persistence: dual-layer JSON and Excel storage, plan CRUD in Enterprise & Operator portals, entity-too-large fix, and real-time sync
</commit_message>
<xml_diff>
--- a/shared/CallerID-Database.xlsx
+++ b/shared/CallerID-Database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="187">
   <si>
     <t>packageId</t>
   </si>
@@ -49,36 +49,39 @@
     <t>abc bank</t>
   </si>
   <si>
+    <t>removed</t>
+  </si>
+  <si>
+    <t>2026-10-20T04:03:43.441Z</t>
+  </si>
+  <si>
+    <t>PKG-ba56e9e1</t>
+  </si>
+  <si>
+    <t>pro plan</t>
+  </si>
+  <si>
+    <t>2026-10-20T04:06:27.852Z</t>
+  </si>
+  <si>
+    <t>PKG-77a27018</t>
+  </si>
+  <si>
+    <t>Bank Standard</t>
+  </si>
+  <si>
+    <t>2026-10-24T05:54:54.254Z</t>
+  </si>
+  <si>
+    <t>PKG-42673541</t>
+  </si>
+  <si>
+    <t>basic 2</t>
+  </si>
+  <si>
     <t>published</t>
   </si>
   <si>
-    <t>2026-10-20T04:03:43.441Z</t>
-  </si>
-  <si>
-    <t>PKG-ba56e9e1</t>
-  </si>
-  <si>
-    <t>pro plan</t>
-  </si>
-  <si>
-    <t>2026-10-20T04:06:27.852Z</t>
-  </si>
-  <si>
-    <t>PKG-77a27018</t>
-  </si>
-  <si>
-    <t>Bank Standard</t>
-  </si>
-  <si>
-    <t>2026-10-24T05:54:54.254Z</t>
-  </si>
-  <si>
-    <t>PKG-42673541</t>
-  </si>
-  <si>
-    <t>basic 2</t>
-  </si>
-  <si>
     <t>2026-10-24T06:30:44.840Z</t>
   </si>
   <si>
@@ -91,6 +94,51 @@
     <t>2026-10-26T07:15:17.955Z</t>
   </si>
   <si>
+    <t>PKG-319e1215</t>
+  </si>
+  <si>
+    <t>Test Plan</t>
+  </si>
+  <si>
+    <t>2026-10-26T13:42:49.646Z</t>
+  </si>
+  <si>
+    <t>PKG-f82e3f8a</t>
+  </si>
+  <si>
+    <t>Enterprise Ultra 2026 - Updated</t>
+  </si>
+  <si>
+    <t>2026-10-26T14:06:42.043Z</t>
+  </si>
+  <si>
+    <t>PKG-perm-test-01</t>
+  </si>
+  <si>
+    <t>Permanent Enterprise Plan</t>
+  </si>
+  <si>
+    <t>2026-10-26T14:09:25.163Z</t>
+  </si>
+  <si>
+    <t>PKG-6041e02d</t>
+  </si>
+  <si>
+    <t>HTTP Test Plan</t>
+  </si>
+  <si>
+    <t>2026-10-26T14:35:16.316Z</t>
+  </si>
+  <si>
+    <t>PKG-6228dcb7</t>
+  </si>
+  <si>
+    <t>basic</t>
+  </si>
+  <si>
+    <t>2026-10-26T14:41:17.414Z</t>
+  </si>
+  <si>
     <t>requestId</t>
   </si>
   <si>
@@ -202,12 +250,18 @@
     <t>always yours</t>
   </si>
   <si>
-    <t>pending</t>
-  </si>
-  <si>
     <t>2026-10-24T07:21:00.000Z</t>
   </si>
   <si>
+    <t>REQ-12205d18</t>
+  </si>
+  <si>
+    <t>FILE-35c74464</t>
+  </si>
+  <si>
+    <t>2026-10-26T14:42:41.793Z</t>
+  </si>
+  <si>
     <t>numberId</t>
   </si>
   <si>
@@ -400,6 +454,51 @@
     <t>NUM-56b7b005</t>
   </si>
   <si>
+    <t>NUM-8155e67c</t>
+  </si>
+  <si>
+    <t>+639171434567</t>
+  </si>
+  <si>
+    <t>+63 917 143 4567</t>
+  </si>
+  <si>
+    <t>NUM-8ca0bd09</t>
+  </si>
+  <si>
+    <t>+639171234566</t>
+  </si>
+  <si>
+    <t>+63 917 123 4566</t>
+  </si>
+  <si>
+    <t>NUM-f4694952</t>
+  </si>
+  <si>
+    <t>+63281237567</t>
+  </si>
+  <si>
+    <t>+63 2 8123 7567</t>
+  </si>
+  <si>
+    <t>NUM-c49fa680</t>
+  </si>
+  <si>
+    <t>+639185558101</t>
+  </si>
+  <si>
+    <t>+63 918 555 8101</t>
+  </si>
+  <si>
+    <t>NUM-731aafb6</t>
+  </si>
+  <si>
+    <t>+631800101234967</t>
+  </si>
+  <si>
+    <t>+63 1800 10123 4967</t>
+  </si>
+  <si>
     <t>fileId</t>
   </si>
   <si>
@@ -470,6 +569,12 @@
   </si>
   <si>
     <t>storage/logos/FILE-aac88032.png</t>
+  </si>
+  <si>
+    <t>FILE-35c74464.png</t>
+  </si>
+  <si>
+    <t>storage/logos/FILE-35c74464.png</t>
   </si>
 </sst>
 </file>
@@ -695,6 +800,45 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>13999</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>17999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="533400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -840,6 +984,45 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>13999</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>17999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="533400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1181,7 +1364,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="14" customWidth="1"/>
@@ -1328,18 +1511,18 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="I5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -1357,10 +1540,155 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2">
+        <v>999</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
         <v>11</v>
       </c>
-      <c r="I6" t="s">
-        <v>24</v>
+      <c r="I7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8">
+        <v>30</v>
+      </c>
+      <c r="D8" s="2">
+        <v>35000</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9">
+        <v>50</v>
+      </c>
+      <c r="D9" s="2">
+        <v>45000</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10">
+        <v>15</v>
+      </c>
+      <c r="D10" s="2">
+        <v>18000</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" s="2">
+        <v>15000</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1371,7 +1699,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="14" customWidth="1"/>
@@ -1383,13 +1711,13 @@
   <sheetData>
     <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
@@ -1398,57 +1726,57 @@
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="H2" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="I2">
         <v>5</v>
@@ -1463,33 +1791,33 @@
         <v>16800</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="G3" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="H3" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="I3">
         <v>4</v>
@@ -1504,33 +1832,33 @@
         <v>22400</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F4" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="H4" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="I4">
         <v>5</v>
@@ -1545,33 +1873,33 @@
         <v>16800</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" t="s">
         <v>57</v>
-      </c>
-      <c r="G5" t="s">
-        <v>58</v>
-      </c>
-      <c r="H5" t="s">
-        <v>41</v>
       </c>
       <c r="I5">
         <v>5</v>
@@ -1586,33 +1914,33 @@
         <v>16800</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="G6" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="H6" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="I6">
         <v>5</v>
@@ -1625,6 +1953,47 @@
       </c>
       <c r="L6">
         <v>16800</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" t="s">
+        <v>81</v>
+      </c>
+      <c r="H7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7" s="2">
+        <v>15000</v>
+      </c>
+      <c r="K7" s="2">
+        <v>1800</v>
+      </c>
+      <c r="L7" s="2">
+        <v>16800</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1633,16 +2002,17 @@
     <hyperlink ref="M3" r:id="rId2"/>
     <hyperlink ref="M4" r:id="rId3"/>
     <hyperlink ref="M5" r:id="rId4"/>
+    <hyperlink ref="M7" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="14" customWidth="1"/>
@@ -1652,25 +2022,25 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -1681,698 +2051,843 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="F2" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I2" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I3" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E4" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="G4" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I4" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="E5" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="F5" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="G5" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H5" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D6" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="E6" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="H6" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G7" t="s">
         <v>91</v>
       </c>
-      <c r="B7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" t="s">
-        <v>78</v>
-      </c>
-      <c r="E7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F7" t="s">
-        <v>93</v>
-      </c>
-      <c r="G7" t="s">
-        <v>73</v>
-      </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="I7" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E8" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="F8" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H8" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="I8" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="E9" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="F9" t="s">
+        <v>117</v>
+      </c>
+      <c r="G9" t="s">
         <v>99</v>
       </c>
-      <c r="G9" t="s">
-        <v>81</v>
-      </c>
       <c r="H9" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="I9" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="E10" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="F10" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H10" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="I10" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H11" t="s">
+        <v>62</v>
+      </c>
+      <c r="I11" t="s">
         <v>70</v>
-      </c>
-      <c r="E11" t="s">
-        <v>71</v>
-      </c>
-      <c r="F11" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" t="s">
-        <v>73</v>
-      </c>
-      <c r="H11" t="s">
-        <v>46</v>
-      </c>
-      <c r="I11" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E12" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" t="s">
+        <v>94</v>
+      </c>
+      <c r="G12" t="s">
+        <v>91</v>
+      </c>
+      <c r="H12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" t="s">
         <v>70</v>
-      </c>
-      <c r="E12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F12" t="s">
-        <v>76</v>
-      </c>
-      <c r="G12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I12" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D13" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="G13" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H13" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="I13" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D14" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="F14" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H14" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="I14" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" t="s">
+        <v>105</v>
+      </c>
+      <c r="E15" t="s">
+        <v>106</v>
+      </c>
+      <c r="F15" t="s">
         <v>107</v>
       </c>
-      <c r="B15" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E15" t="s">
-        <v>88</v>
-      </c>
-      <c r="F15" t="s">
-        <v>89</v>
-      </c>
       <c r="G15" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="H15" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="I15" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E16" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="F16" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="G16" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H16" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I16" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>129</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="F17" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="G17" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H17" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I17" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D18" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E18" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="F18" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="G18" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H18" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I18" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D19" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="E19" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="F19" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="G19" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H19" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I19" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D20" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="E20" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="F20" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="G20" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="H20" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="I20" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D21" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E21" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="F21" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H21" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="I21" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D22" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E22" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="F22" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="G22" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H22" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="I22" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D23" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" t="s">
+        <v>97</v>
+      </c>
+      <c r="F23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H23" t="s">
+        <v>54</v>
+      </c>
+      <c r="I23" t="s">
         <v>78</v>
-      </c>
-      <c r="E23" t="s">
-        <v>79</v>
-      </c>
-      <c r="F23" t="s">
-        <v>80</v>
-      </c>
-      <c r="G23" t="s">
-        <v>81</v>
-      </c>
-      <c r="H23" t="s">
-        <v>62</v>
-      </c>
-      <c r="I23" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="B24" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="E24" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="F24" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H24" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="I24" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D25" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="E25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" t="s">
+        <v>107</v>
+      </c>
+      <c r="G25" t="s">
+        <v>108</v>
+      </c>
+      <c r="H25" t="s">
+        <v>54</v>
+      </c>
+      <c r="I25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>146</v>
+      </c>
+      <c r="B26" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" t="s">
         <v>88</v>
       </c>
-      <c r="F25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H25" t="s">
+      <c r="E26" t="s">
+        <v>147</v>
+      </c>
+      <c r="F26" t="s">
+        <v>148</v>
+      </c>
+      <c r="G26" t="s">
+        <v>91</v>
+      </c>
+      <c r="H26" t="s">
         <v>62</v>
       </c>
-      <c r="I25" t="s">
-        <v>63</v>
+      <c r="I26" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" t="s">
+        <v>88</v>
+      </c>
+      <c r="E27" t="s">
+        <v>150</v>
+      </c>
+      <c r="F27" t="s">
+        <v>151</v>
+      </c>
+      <c r="G27" t="s">
+        <v>91</v>
+      </c>
+      <c r="H27" t="s">
+        <v>62</v>
+      </c>
+      <c r="I27" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>152</v>
+      </c>
+      <c r="B28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" t="s">
+        <v>154</v>
+      </c>
+      <c r="G28" t="s">
+        <v>99</v>
+      </c>
+      <c r="H28" t="s">
+        <v>62</v>
+      </c>
+      <c r="I28" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>155</v>
+      </c>
+      <c r="B29" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" t="s">
+        <v>101</v>
+      </c>
+      <c r="E29" t="s">
+        <v>156</v>
+      </c>
+      <c r="F29" t="s">
+        <v>157</v>
+      </c>
+      <c r="G29" t="s">
+        <v>91</v>
+      </c>
+      <c r="H29" t="s">
+        <v>62</v>
+      </c>
+      <c r="I29" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" t="s">
+        <v>105</v>
+      </c>
+      <c r="E30" t="s">
+        <v>159</v>
+      </c>
+      <c r="F30" t="s">
+        <v>160</v>
+      </c>
+      <c r="G30" t="s">
+        <v>108</v>
+      </c>
+      <c r="H30" t="s">
+        <v>62</v>
+      </c>
+      <c r="I30" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2383,7 +2898,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2395,180 +2910,215 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>162</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>163</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>131</v>
+        <v>164</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>133</v>
+        <v>166</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>134</v>
+        <v>167</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>136</v>
+        <v>169</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>137</v>
+        <v>170</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="D2" t="s">
-        <v>139</v>
+        <v>172</v>
       </c>
       <c r="E2" t="s">
-        <v>140</v>
+        <v>173</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="G2" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="H2">
         <v>869308</v>
       </c>
       <c r="I2" t="s">
-        <v>142</v>
+        <v>175</v>
       </c>
       <c r="J2" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="K2" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="D3" t="s">
-        <v>144</v>
+        <v>177</v>
       </c>
       <c r="E3" t="s">
-        <v>145</v>
+        <v>178</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="G3" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="H3">
         <v>869308</v>
       </c>
       <c r="I3" t="s">
-        <v>142</v>
+        <v>175</v>
       </c>
       <c r="J3" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="K3" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>146</v>
+        <v>179</v>
       </c>
       <c r="D4" t="s">
-        <v>147</v>
+        <v>180</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>181</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="G4" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="H4">
         <v>12539</v>
       </c>
       <c r="I4" t="s">
-        <v>149</v>
+        <v>182</v>
       </c>
       <c r="J4" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="K4" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="D5" t="s">
-        <v>150</v>
+        <v>183</v>
       </c>
       <c r="E5" t="s">
-        <v>151</v>
+        <v>184</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="G5" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="H5">
         <v>869308</v>
       </c>
       <c r="I5" t="s">
-        <v>142</v>
+        <v>175</v>
       </c>
       <c r="J5" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="K5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E6" t="s">
+        <v>186</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>58</v>
+      </c>
+      <c r="G6" t="s">
+        <v>174</v>
+      </c>
+      <c r="H6">
+        <v>869308</v>
+      </c>
+      <c r="I6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J6" t="s">
+        <v>176</v>
+      </c>
+      <c r="K6" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2577,9 +3127,10 @@
     <hyperlink ref="F3" r:id="rId2"/>
     <hyperlink ref="F4" r:id="rId3"/>
     <hyperlink ref="F5" r:id="rId4"/>
+    <hyperlink ref="F6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement Subscription & Brand Requests Management, Operator review workflow, Android caller screen, and logo persistence bug fix
</commit_message>
<xml_diff>
--- a/shared/CallerID-Database.xlsx
+++ b/shared/CallerID-Database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="207">
   <si>
     <t>packageId</t>
   </si>
@@ -169,6 +169,12 @@
     <t>preview</t>
   </si>
   <si>
+    <t>callReason</t>
+  </si>
+  <si>
+    <t>remarks</t>
+  </si>
+  <si>
     <t>REQ-6b079415</t>
   </si>
   <si>
@@ -262,6 +268,27 @@
     <t>2026-10-26T14:42:41.793Z</t>
   </si>
   <si>
+    <t>REQ-31bb3367</t>
+  </si>
+  <si>
+    <t>Metropolitan Bank &amp; Trust</t>
+  </si>
+  <si>
+    <t>Diwali Festive Offers &amp; Rewards</t>
+  </si>
+  <si>
+    <t>FILE-93e8a7b6</t>
+  </si>
+  <si>
+    <t>2026-10-27T09:12:55.720Z</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Click "Open file" to view</t>
+  </si>
+  <si>
     <t>numberId</t>
   </si>
   <si>
@@ -499,6 +526,24 @@
     <t>+63 1800 10123 4967</t>
   </si>
   <si>
+    <t>NUM-4611f9f9</t>
+  </si>
+  <si>
+    <t>+639171234501</t>
+  </si>
+  <si>
+    <t>+63 917 123 4501</t>
+  </si>
+  <si>
+    <t>NUM-30b7f79f</t>
+  </si>
+  <si>
+    <t>+639171234502</t>
+  </si>
+  <si>
+    <t>+63 917 123 4502</t>
+  </si>
+  <si>
     <t>fileId</t>
   </si>
   <si>
@@ -575,6 +620,21 @@
   </si>
   <si>
     <t>storage/logos/FILE-35c74464.png</t>
+  </si>
+  <si>
+    <t>metrobank.svg</t>
+  </si>
+  <si>
+    <t>FILE-93e8a7b6.svg</t>
+  </si>
+  <si>
+    <t>storage/logos/FILE-93e8a7b6.svg</t>
+  </si>
+  <si>
+    <t>image/svg+xml</t>
+  </si>
+  <si>
+    <t>90306b61bae0b34c5dd51049cf230b2e36a2604c39f832665e9207813b066a75</t>
   </si>
 </sst>
 </file>
@@ -1699,17 +1759,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="14" width="14" customWidth="1"/>
+    <col min="11" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
@@ -1752,31 +1812,37 @@
       <c r="N1" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I2">
         <v>5</v>
@@ -1791,33 +1857,33 @@
         <v>16800</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I3">
         <v>4</v>
@@ -1832,33 +1898,33 @@
         <v>22400</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I4">
         <v>5</v>
@@ -1873,33 +1939,33 @@
         <v>16800</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I5">
         <v>5</v>
@@ -1914,33 +1980,33 @@
         <v>16800</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I6">
         <v>5</v>
@@ -1957,28 +2023,28 @@
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B7" t="s">
         <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -1993,7 +2059,57 @@
         <v>16800</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H8" t="s">
+        <v>89</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8" s="2">
+        <v>15000</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1800</v>
+      </c>
+      <c r="L8" s="2">
+        <v>16800</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="N8" t="s">
+        <v>90</v>
+      </c>
+      <c r="O8" t="s">
+        <v>86</v>
+      </c>
+      <c r="P8" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2003,16 +2119,17 @@
     <hyperlink ref="M4" r:id="rId3"/>
     <hyperlink ref="M5" r:id="rId4"/>
     <hyperlink ref="M7" r:id="rId5"/>
+    <hyperlink ref="M8" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="14" customWidth="1"/>
@@ -2022,7 +2139,7 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>41</v>
@@ -2031,16 +2148,16 @@
         <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -2051,843 +2168,901 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="G2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="G3" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="F4" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G4" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F5" t="s">
+        <v>112</v>
+      </c>
+      <c r="G5" t="s">
         <v>100</v>
       </c>
-      <c r="B5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" t="s">
-        <v>101</v>
-      </c>
-      <c r="E5" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" t="s">
-        <v>103</v>
-      </c>
-      <c r="G5" t="s">
-        <v>91</v>
-      </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D6" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E6" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="G6" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D7" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="F7" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="F8" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E9" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="F9" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="G9" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E10" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="F10" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="G10" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E11" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="F11" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="G11" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E12" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="G12" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E13" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="F13" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G13" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="F14" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="G14" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I14" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D15" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F15" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="G15" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C16" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E16" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="F16" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="G16" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H16" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E17" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F17" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="G17" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H17" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D18" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E18" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="F18" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="G18" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H18" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D19" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E19" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="F19" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G19" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D20" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E20" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="F20" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="G20" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H20" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E21" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="F21" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="G21" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D22" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E22" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F22" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="G22" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H22" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D23" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E23" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="F23" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G23" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H23" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I23" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D24" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E24" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="F24" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="G24" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H24" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I24" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D25" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E25" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F25" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="G25" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E26" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="F26" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="G26" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H26" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I26" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D27" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E27" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="F27" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="G27" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H27" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C28" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D28" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E28" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="F28" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="G28" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H28" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I28" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="B29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D29" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E29" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="F29" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G29" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I29" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D30" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E30" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="F30" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="G30" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H30" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I30" t="s">
-        <v>81</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>170</v>
+      </c>
+      <c r="B31" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" t="s">
+        <v>85</v>
+      </c>
+      <c r="D31" t="s">
+        <v>89</v>
+      </c>
+      <c r="E31" t="s">
+        <v>171</v>
+      </c>
+      <c r="F31" t="s">
+        <v>172</v>
+      </c>
+      <c r="G31" t="s">
+        <v>100</v>
+      </c>
+      <c r="H31" t="s">
+        <v>64</v>
+      </c>
+      <c r="I31" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>173</v>
+      </c>
+      <c r="B32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" t="s">
+        <v>85</v>
+      </c>
+      <c r="D32" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" t="s">
+        <v>174</v>
+      </c>
+      <c r="F32" t="s">
+        <v>175</v>
+      </c>
+      <c r="G32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I32" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2898,7 +3073,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2910,37 +3085,37 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>50</v>
@@ -2948,177 +3123,215 @@
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="D2" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="E2" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="H2">
         <v>869308</v>
       </c>
       <c r="I2" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="J2" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="K2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="D3" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="E3" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G3" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="H3">
         <v>869308</v>
       </c>
       <c r="I3" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="J3" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="K3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="D4" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="E4" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="H4">
         <v>12539</v>
       </c>
       <c r="I4" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="J4" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="K4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" t="s">
         <v>73</v>
       </c>
-      <c r="B5" t="s">
-        <v>71</v>
-      </c>
       <c r="C5" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="D5" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="E5" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="H5">
         <v>869308</v>
       </c>
       <c r="I5" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="J5" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="K5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="D6" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="E6" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G6" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="H6">
         <v>869308</v>
       </c>
       <c r="I6" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="J6" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="K6" t="s">
-        <v>81</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" t="s">
+        <v>202</v>
+      </c>
+      <c r="D7" t="s">
+        <v>203</v>
+      </c>
+      <c r="E7" t="s">
+        <v>204</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>205</v>
+      </c>
+      <c r="H7">
+        <v>115</v>
+      </c>
+      <c r="I7" t="s">
+        <v>206</v>
+      </c>
+      <c r="J7" t="s">
+        <v>191</v>
+      </c>
+      <c r="K7" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -3128,9 +3341,10 @@
     <hyperlink ref="F4" r:id="rId3"/>
     <hyperlink ref="F5" r:id="rId4"/>
     <hyperlink ref="F6" r:id="rId5"/>
+    <hyperlink ref="F7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix mutual recursion between parseAndValidateNumbers and updateLivePreview
</commit_message>
<xml_diff>
--- a/shared/CallerID-Database.xlsx
+++ b/shared/CallerID-Database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="213">
   <si>
     <t>packageId</t>
   </si>
@@ -43,6 +43,15 @@
     <t>createdAt</t>
   </si>
   <si>
+    <t>duration</t>
+  </si>
+  <si>
+    <t>brandedCalls</t>
+  </si>
+  <si>
+    <t>callReason</t>
+  </si>
+  <si>
     <t>PKG-ea45b292</t>
   </si>
   <si>
@@ -139,6 +148,18 @@
     <t>2026-10-26T14:41:17.414Z</t>
   </si>
   <si>
+    <t>PKG-2e970224</t>
+  </si>
+  <si>
+    <t>basic 3</t>
+  </si>
+  <si>
+    <t>2026-10-27T09:23:04.803Z</t>
+  </si>
+  <si>
+    <t>30 Days</t>
+  </si>
+  <si>
     <t>requestId</t>
   </si>
   <si>
@@ -167,9 +188,6 @@
   </si>
   <si>
     <t>preview</t>
-  </si>
-  <si>
-    <t>callReason</t>
   </si>
   <si>
     <t>remarks</t>
@@ -1424,15 +1442,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="14" customWidth="1"/>
+    <col min="8" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1460,13 +1480,22 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -1484,18 +1513,18 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>5</v>
@@ -1513,18 +1542,18 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>5</v>
@@ -1542,18 +1571,18 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>5</v>
@@ -1571,18 +1600,18 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -1600,18 +1629,18 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C7">
         <v>10</v>
@@ -1629,18 +1658,18 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C8">
         <v>30</v>
@@ -1658,18 +1687,18 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C9">
         <v>50</v>
@@ -1687,18 +1716,18 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I9" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C10">
         <v>15</v>
@@ -1716,18 +1745,18 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I10" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C11">
         <v>5</v>
@@ -1745,10 +1774,48 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I11" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2">
+        <v>15000</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" t="s">
+        <v>46</v>
+      </c>
+      <c r="J12" t="s">
+        <v>47</v>
+      </c>
+      <c r="K12">
+        <v>50000</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1771,13 +1838,13 @@
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
@@ -1786,63 +1853,63 @@
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="G2" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I2">
         <v>5</v>
@@ -1857,33 +1924,33 @@
         <v>16800</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="G3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I3">
         <v>4</v>
@@ -1898,33 +1965,33 @@
         <v>22400</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" t="s">
         <v>70</v>
       </c>
-      <c r="E4" t="s">
-        <v>64</v>
-      </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G4" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I4">
         <v>5</v>
@@ -1939,33 +2006,33 @@
         <v>16800</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="H5" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I5">
         <v>5</v>
@@ -1980,33 +2047,33 @@
         <v>16800</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H6" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I6">
         <v>5</v>
@@ -2023,28 +2090,28 @@
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F7" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G7" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -2059,33 +2126,33 @@
         <v>16800</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D8" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G8" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="H8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="I8">
         <v>2</v>
@@ -2100,16 +2167,16 @@
         <v>16800</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="N8" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="O8" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="P8" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -2139,25 +2206,25 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -2168,901 +2235,901 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="F3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H3" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="G4" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H4" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I4" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E5" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H5" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I5" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E6" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="G6" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E7" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="F7" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="G7" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D8" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="F8" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="G8" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D9" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F9" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I9" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F10" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="G10" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I10" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E11" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F11" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G11" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I11" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E12" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="F12" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G12" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H12" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I12" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E13" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F13" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="G13" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H13" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I13" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D14" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E14" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F14" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G14" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H14" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I14" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E15" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F15" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="G15" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H15" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I15" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C16" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D16" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E16" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="F16" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G16" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H16" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I16" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D17" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E17" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="F17" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="G17" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H17" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I17" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D18" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E18" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="F18" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="G18" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H18" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I18" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D19" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E19" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="F19" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="G19" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H19" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I19" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D20" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E20" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="F20" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="G20" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H20" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I20" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D21" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E21" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F21" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G21" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H21" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I21" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E22" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="F22" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G22" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H22" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I22" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B23" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D23" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E23" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F23" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="G23" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H23" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I23" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D24" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E24" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F24" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G24" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H24" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I24" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B25" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D25" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E25" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F25" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="G25" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H25" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I25" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B26" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C26" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D26" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E26" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="F26" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="G26" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H26" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I26" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B27" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C27" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E27" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="F27" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G27" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H27" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I27" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B28" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D28" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E28" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F28" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="G28" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H28" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I28" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B29" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C29" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D29" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E29" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="F29" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="G29" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H29" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I29" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B30" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C30" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D30" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E30" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="F30" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="G30" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H30" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I30" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B31" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C31" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D31" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E31" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="F31" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="G31" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H31" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I31" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B32" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C32" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D32" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E32" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="F32" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="G32" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H32" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I32" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -3085,253 +3152,253 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D2" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="E2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="G2" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="H2">
         <v>869308</v>
       </c>
       <c r="I2" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="J2" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K2" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="G3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="H3">
         <v>869308</v>
       </c>
       <c r="I3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="J3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" t="s">
         <v>195</v>
-      </c>
-      <c r="E4" t="s">
-        <v>196</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G4" t="s">
-        <v>189</v>
       </c>
       <c r="H4">
         <v>12539</v>
       </c>
       <c r="I4" t="s">
+        <v>203</v>
+      </c>
+      <c r="J4" t="s">
         <v>197</v>
       </c>
-      <c r="J4" t="s">
-        <v>191</v>
-      </c>
       <c r="K4" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D5" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="E5" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="G5" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="H5">
         <v>869308</v>
       </c>
       <c r="I5" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="J5" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K5" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C6" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="E6" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="G6" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="H6">
         <v>869308</v>
       </c>
       <c r="I6" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="J6" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K6" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="D7" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E7" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="G7" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="H7">
         <v>115</v>
       </c>
       <c r="I7" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K7" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="L7" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update test request database state
</commit_message>
<xml_diff>
--- a/shared/CallerID-Database.xlsx
+++ b/shared/CallerID-Database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="216">
   <si>
     <t>packageId</t>
   </si>
@@ -158,6 +158,15 @@
   </si>
   <si>
     <t>30 Days</t>
+  </si>
+  <si>
+    <t>PKG-69c8e7d6</t>
+  </si>
+  <si>
+    <t>VIP Plan</t>
+  </si>
+  <si>
+    <t>2026-10-27T09:33:52.890Z</t>
   </si>
   <si>
     <t>requestId</t>
@@ -1442,7 +1451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="14" customWidth="1"/>
@@ -1815,6 +1824,44 @@
         <v>50000</v>
       </c>
       <c r="L12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13">
+        <v>50</v>
+      </c>
+      <c r="D13" s="2">
+        <v>25000</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" t="s">
+        <v>50</v>
+      </c>
+      <c r="J13" t="s">
+        <v>47</v>
+      </c>
+      <c r="K13">
+        <v>50000</v>
+      </c>
+      <c r="L13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1838,13 +1885,13 @@
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
@@ -1853,63 +1900,63 @@
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I2">
         <v>5</v>
@@ -1924,33 +1971,33 @@
         <v>16800</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I3">
         <v>4</v>
@@ -1965,33 +2012,33 @@
         <v>22400</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I4">
         <v>5</v>
@@ -2006,33 +2053,33 @@
         <v>16800</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I5">
         <v>5</v>
@@ -2047,33 +2094,33 @@
         <v>16800</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D6" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I6">
         <v>5</v>
@@ -2090,28 +2137,28 @@
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
         <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D7" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G7" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H7" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -2126,33 +2173,33 @@
         <v>16800</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
         <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D8" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G8" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I8">
         <v>2</v>
@@ -2167,16 +2214,16 @@
         <v>16800</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="N8" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="O8" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P8" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2206,25 +2253,25 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -2235,901 +2282,901 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" t="s">
         <v>109</v>
       </c>
-      <c r="G3" t="s">
-        <v>106</v>
-      </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="G6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I7" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D8" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F8" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G8" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F9" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="G9" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E10" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H10" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F11" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G11" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D12" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E12" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F12" t="s">
+        <v>112</v>
+      </c>
+      <c r="G12" t="s">
         <v>109</v>
       </c>
-      <c r="G12" t="s">
-        <v>106</v>
-      </c>
       <c r="H12" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F13" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G13" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H13" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E14" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F14" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G14" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H14" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E15" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F15" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="G15" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H15" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D16" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E16" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F16" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G16" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I16" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E17" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F17" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H17" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I17" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E18" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F18" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G18" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H18" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I18" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B19" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D19" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E19" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F19" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="G19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H19" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I19" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E20" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F20" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="G20" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I20" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D21" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E21" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F21" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G21" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H21" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I21" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B22" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C22" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E22" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F22" t="s">
+        <v>112</v>
+      </c>
+      <c r="G22" t="s">
         <v>109</v>
       </c>
-      <c r="G22" t="s">
-        <v>106</v>
-      </c>
       <c r="H22" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I22" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B23" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D23" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E23" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F23" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G23" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H23" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I23" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D24" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F24" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G24" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H24" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I24" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E25" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F25" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="G25" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H25" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I25" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B26" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" t="s">
         <v>87</v>
       </c>
-      <c r="C26" t="s">
-        <v>84</v>
-      </c>
       <c r="D26" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E26" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F26" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G26" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H26" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I26" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B27" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" t="s">
         <v>87</v>
       </c>
-      <c r="C27" t="s">
-        <v>84</v>
-      </c>
       <c r="D27" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E27" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F27" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G27" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H27" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I27" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" t="s">
         <v>87</v>
       </c>
-      <c r="C28" t="s">
-        <v>84</v>
-      </c>
       <c r="D28" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E28" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F28" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G28" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H28" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I28" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B29" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" t="s">
         <v>87</v>
       </c>
-      <c r="C29" t="s">
-        <v>84</v>
-      </c>
       <c r="D29" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F29" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="G29" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H29" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I29" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B30" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" t="s">
         <v>87</v>
       </c>
-      <c r="C30" t="s">
-        <v>84</v>
-      </c>
       <c r="D30" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E30" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F30" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G30" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H30" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I30" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C31" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D31" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E31" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F31" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G31" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H31" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I31" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C32" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D32" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F32" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G32" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H32" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I32" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -3152,253 +3199,253 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H2">
         <v>869308</v>
       </c>
       <c r="I2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="K2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D3" t="s">
+        <v>201</v>
+      </c>
+      <c r="E3" t="s">
+        <v>202</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" t="s">
         <v>198</v>
-      </c>
-      <c r="E3" t="s">
-        <v>199</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" t="s">
-        <v>195</v>
       </c>
       <c r="H3">
         <v>869308</v>
       </c>
       <c r="I3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="K3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" t="s">
         <v>77</v>
       </c>
-      <c r="B4" t="s">
-        <v>74</v>
-      </c>
       <c r="C4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D4" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E4" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G4" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H4">
         <v>12539</v>
       </c>
       <c r="I4" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="J4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="K4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H5">
         <v>869308</v>
       </c>
       <c r="I5" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J5" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="K5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D6" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="E6" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G6" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H6">
         <v>869308</v>
       </c>
       <c r="I6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="K6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
         <v>93</v>
       </c>
-      <c r="B7" t="s">
-        <v>90</v>
-      </c>
       <c r="C7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="H7">
         <v>115</v>
       </c>
       <c r="I7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="J7" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="K7" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="L7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
simplify: single Fill Number button, remove dice/bulk/paste options
</commit_message>
<xml_diff>
--- a/shared/CallerID-Database.xlsx
+++ b/shared/CallerID-Database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="239">
   <si>
     <t>packageId</t>
   </si>
@@ -316,6 +316,27 @@
     <t>Click "Open file" to view</t>
   </si>
   <si>
+    <t>REQ-7785e6bc</t>
+  </si>
+  <si>
+    <t>Metropolitan Bank</t>
+  </si>
+  <si>
+    <t>Exclusive Diwali Offer</t>
+  </si>
+  <si>
+    <t>pending</t>
+  </si>
+  <si>
+    <t>FILE-3204d32b</t>
+  </si>
+  <si>
+    <t>2026-10-27T10:51:07.925Z</t>
+  </si>
+  <si>
+    <t>Customer Service</t>
+  </si>
+  <si>
     <t>numberId</t>
   </si>
   <si>
@@ -334,9 +355,6 @@
     <t>NUM-3c3cf48e</t>
   </si>
   <si>
-    <t>Customer Service</t>
-  </si>
-  <si>
     <t>+639171234567</t>
   </si>
   <si>
@@ -571,6 +589,51 @@
     <t>+63 917 123 4502</t>
   </si>
   <si>
+    <t>NUM-7b923a91</t>
+  </si>
+  <si>
+    <t>+639398386747</t>
+  </si>
+  <si>
+    <t>+63 939 838 6747</t>
+  </si>
+  <si>
+    <t>NUM-8f6f703f</t>
+  </si>
+  <si>
+    <t>+639226672114</t>
+  </si>
+  <si>
+    <t>+63 922 667 2114</t>
+  </si>
+  <si>
+    <t>NUM-ba788fab</t>
+  </si>
+  <si>
+    <t>+639218448404</t>
+  </si>
+  <si>
+    <t>+63 921 844 8404</t>
+  </si>
+  <si>
+    <t>NUM-aa7ecee1</t>
+  </si>
+  <si>
+    <t>+639279868730</t>
+  </si>
+  <si>
+    <t>+63 927 986 8730</t>
+  </si>
+  <si>
+    <t>NUM-727bfe85</t>
+  </si>
+  <si>
+    <t>+639192216074</t>
+  </si>
+  <si>
+    <t>+63 919 221 6074</t>
+  </si>
+  <si>
     <t>fileId</t>
   </si>
   <si>
@@ -662,6 +725,12 @@
   </si>
   <si>
     <t>90306b61bae0b34c5dd51049cf230b2e36a2604c39f832665e9207813b066a75</t>
+  </si>
+  <si>
+    <t>FILE-3204d32b.png</t>
+  </si>
+  <si>
+    <t>storage/logos/FILE-3204d32b.png</t>
   </si>
 </sst>
 </file>
@@ -926,6 +995,45 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>13999</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>17999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="533400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1098,6 +1206,45 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>13999</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>17999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="533400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
@@ -1873,7 +2020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="14" customWidth="1"/>
@@ -2226,6 +2373,53 @@
         <v>64</v>
       </c>
     </row>
+    <row r="9" ht="48" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H9" t="s">
+        <v>106</v>
+      </c>
+      <c r="I9">
+        <v>5</v>
+      </c>
+      <c r="J9" s="2">
+        <v>15000</v>
+      </c>
+      <c r="K9" s="2">
+        <v>1800</v>
+      </c>
+      <c r="L9" s="2">
+        <v>16800</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="O9" t="s">
+        <v>102</v>
+      </c>
+      <c r="P9" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1"/>
@@ -2234,16 +2428,17 @@
     <hyperlink ref="M5" r:id="rId4"/>
     <hyperlink ref="M7" r:id="rId5"/>
     <hyperlink ref="M8" r:id="rId6"/>
+    <hyperlink ref="M9" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="14" customWidth="1"/>
@@ -2253,7 +2448,7 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>51</v>
@@ -2262,16 +2457,16 @@
         <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -2282,7 +2477,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>62</v>
@@ -2294,13 +2489,13 @@
         <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="F2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="G2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H2" t="s">
         <v>65</v>
@@ -2311,7 +2506,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B3" t="s">
         <v>62</v>
@@ -2323,13 +2518,13 @@
         <v>106</v>
       </c>
       <c r="E3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G3" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H3" t="s">
         <v>65</v>
@@ -2340,7 +2535,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B4" t="s">
         <v>62</v>
@@ -2349,16 +2544,16 @@
         <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E4" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F4" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="G4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H4" t="s">
         <v>65</v>
@@ -2369,7 +2564,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
         <v>62</v>
@@ -2378,16 +2573,16 @@
         <v>63</v>
       </c>
       <c r="D5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F5" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="G5" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H5" t="s">
         <v>65</v>
@@ -2398,7 +2593,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B6" t="s">
         <v>62</v>
@@ -2407,16 +2602,16 @@
         <v>63</v>
       </c>
       <c r="D6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E6" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G6" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H6" t="s">
         <v>65</v>
@@ -2427,7 +2622,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B7" t="s">
         <v>70</v>
@@ -2436,16 +2631,16 @@
         <v>71</v>
       </c>
       <c r="D7" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E7" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="G7" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H7" t="s">
         <v>73</v>
@@ -2456,7 +2651,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
         <v>70</v>
@@ -2465,16 +2660,16 @@
         <v>71</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E8" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F8" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="G8" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H8" t="s">
         <v>73</v>
@@ -2485,7 +2680,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B9" t="s">
         <v>70</v>
@@ -2494,16 +2689,16 @@
         <v>71</v>
       </c>
       <c r="D9" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E9" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F9" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="G9" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H9" t="s">
         <v>73</v>
@@ -2514,7 +2709,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B10" t="s">
         <v>70</v>
@@ -2523,16 +2718,16 @@
         <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E10" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F10" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H10" t="s">
         <v>73</v>
@@ -2543,7 +2738,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B11" t="s">
         <v>77</v>
@@ -2555,13 +2750,13 @@
         <v>106</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="F11" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="G11" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H11" t="s">
         <v>73</v>
@@ -2572,7 +2767,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B12" t="s">
         <v>77</v>
@@ -2584,13 +2779,13 @@
         <v>106</v>
       </c>
       <c r="E12" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F12" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G12" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H12" t="s">
         <v>73</v>
@@ -2601,7 +2796,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B13" t="s">
         <v>77</v>
@@ -2610,16 +2805,16 @@
         <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E13" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F13" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="G13" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H13" t="s">
         <v>73</v>
@@ -2630,7 +2825,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B14" t="s">
         <v>77</v>
@@ -2639,16 +2834,16 @@
         <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E14" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F14" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="G14" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H14" t="s">
         <v>73</v>
@@ -2659,7 +2854,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B15" t="s">
         <v>77</v>
@@ -2668,16 +2863,16 @@
         <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E15" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F15" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G15" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H15" t="s">
         <v>73</v>
@@ -2688,7 +2883,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B16" t="s">
         <v>82</v>
@@ -2700,13 +2895,13 @@
         <v>106</v>
       </c>
       <c r="E16" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="F16" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="G16" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H16" t="s">
         <v>65</v>
@@ -2717,7 +2912,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B17" t="s">
         <v>82</v>
@@ -2729,13 +2924,13 @@
         <v>106</v>
       </c>
       <c r="E17" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="F17" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="G17" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H17" t="s">
         <v>65</v>
@@ -2746,7 +2941,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B18" t="s">
         <v>82</v>
@@ -2755,16 +2950,16 @@
         <v>83</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E18" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="F18" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="G18" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H18" t="s">
         <v>65</v>
@@ -2775,7 +2970,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B19" t="s">
         <v>82</v>
@@ -2784,16 +2979,16 @@
         <v>83</v>
       </c>
       <c r="D19" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E19" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="F19" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="G19" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H19" t="s">
         <v>65</v>
@@ -2804,7 +2999,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B20" t="s">
         <v>82</v>
@@ -2813,16 +3008,16 @@
         <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E20" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="F20" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="G20" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H20" t="s">
         <v>65</v>
@@ -2833,7 +3028,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B21" t="s">
         <v>86</v>
@@ -2845,13 +3040,13 @@
         <v>106</v>
       </c>
       <c r="E21" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="F21" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="G21" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H21" t="s">
         <v>65</v>
@@ -2862,7 +3057,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B22" t="s">
         <v>86</v>
@@ -2874,13 +3069,13 @@
         <v>106</v>
       </c>
       <c r="E22" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F22" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G22" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H22" t="s">
         <v>65</v>
@@ -2891,7 +3086,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B23" t="s">
         <v>86</v>
@@ -2900,16 +3095,16 @@
         <v>87</v>
       </c>
       <c r="D23" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E23" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F23" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="G23" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H23" t="s">
         <v>65</v>
@@ -2920,7 +3115,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B24" t="s">
         <v>86</v>
@@ -2929,16 +3124,16 @@
         <v>87</v>
       </c>
       <c r="D24" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E24" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F24" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="G24" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H24" t="s">
         <v>65</v>
@@ -2949,7 +3144,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B25" t="s">
         <v>86</v>
@@ -2958,16 +3153,16 @@
         <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E25" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F25" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G25" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H25" t="s">
         <v>65</v>
@@ -2978,7 +3173,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B26" t="s">
         <v>90</v>
@@ -2990,13 +3185,13 @@
         <v>106</v>
       </c>
       <c r="E26" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="F26" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="G26" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H26" t="s">
         <v>73</v>
@@ -3007,7 +3202,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B27" t="s">
         <v>90</v>
@@ -3019,13 +3214,13 @@
         <v>106</v>
       </c>
       <c r="E27" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="F27" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="G27" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H27" t="s">
         <v>73</v>
@@ -3036,7 +3231,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B28" t="s">
         <v>90</v>
@@ -3045,16 +3240,16 @@
         <v>87</v>
       </c>
       <c r="D28" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E28" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="F28" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="G28" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H28" t="s">
         <v>73</v>
@@ -3065,7 +3260,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B29" t="s">
         <v>90</v>
@@ -3074,16 +3269,16 @@
         <v>87</v>
       </c>
       <c r="D29" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E29" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="F29" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="G29" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H29" t="s">
         <v>73</v>
@@ -3094,7 +3289,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B30" t="s">
         <v>90</v>
@@ -3103,16 +3298,16 @@
         <v>87</v>
       </c>
       <c r="D30" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E30" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="F30" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="G30" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H30" t="s">
         <v>73</v>
@@ -3123,7 +3318,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B31" t="s">
         <v>93</v>
@@ -3135,13 +3330,13 @@
         <v>98</v>
       </c>
       <c r="E31" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="F31" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="G31" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H31" t="s">
         <v>73</v>
@@ -3152,7 +3347,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B32" t="s">
         <v>93</v>
@@ -3164,19 +3359,164 @@
         <v>98</v>
       </c>
       <c r="E32" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="F32" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="G32" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H32" t="s">
         <v>73</v>
       </c>
       <c r="I32" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>191</v>
+      </c>
+      <c r="B33" t="s">
+        <v>100</v>
+      </c>
+      <c r="C33" t="s">
+        <v>101</v>
+      </c>
+      <c r="D33" t="s">
+        <v>106</v>
+      </c>
+      <c r="E33" t="s">
+        <v>192</v>
+      </c>
+      <c r="F33" t="s">
+        <v>193</v>
+      </c>
+      <c r="G33" t="s">
+        <v>115</v>
+      </c>
+      <c r="H33" t="s">
+        <v>103</v>
+      </c>
+      <c r="I33" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>194</v>
+      </c>
+      <c r="B34" t="s">
+        <v>100</v>
+      </c>
+      <c r="C34" t="s">
+        <v>101</v>
+      </c>
+      <c r="D34" t="s">
+        <v>106</v>
+      </c>
+      <c r="E34" t="s">
+        <v>195</v>
+      </c>
+      <c r="F34" t="s">
+        <v>196</v>
+      </c>
+      <c r="G34" t="s">
+        <v>115</v>
+      </c>
+      <c r="H34" t="s">
+        <v>103</v>
+      </c>
+      <c r="I34" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>197</v>
+      </c>
+      <c r="B35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C35" t="s">
+        <v>101</v>
+      </c>
+      <c r="D35" t="s">
+        <v>106</v>
+      </c>
+      <c r="E35" t="s">
+        <v>198</v>
+      </c>
+      <c r="F35" t="s">
+        <v>199</v>
+      </c>
+      <c r="G35" t="s">
+        <v>115</v>
+      </c>
+      <c r="H35" t="s">
+        <v>103</v>
+      </c>
+      <c r="I35" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>200</v>
+      </c>
+      <c r="B36" t="s">
+        <v>100</v>
+      </c>
+      <c r="C36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D36" t="s">
+        <v>106</v>
+      </c>
+      <c r="E36" t="s">
+        <v>201</v>
+      </c>
+      <c r="F36" t="s">
+        <v>202</v>
+      </c>
+      <c r="G36" t="s">
+        <v>115</v>
+      </c>
+      <c r="H36" t="s">
+        <v>103</v>
+      </c>
+      <c r="I36" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>203</v>
+      </c>
+      <c r="B37" t="s">
+        <v>100</v>
+      </c>
+      <c r="C37" t="s">
+        <v>101</v>
+      </c>
+      <c r="D37" t="s">
+        <v>106</v>
+      </c>
+      <c r="E37" t="s">
+        <v>204</v>
+      </c>
+      <c r="F37" t="s">
+        <v>205</v>
+      </c>
+      <c r="G37" t="s">
+        <v>115</v>
+      </c>
+      <c r="H37" t="s">
+        <v>103</v>
+      </c>
+      <c r="I37" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -3187,7 +3527,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -3199,37 +3539,37 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>193</v>
+        <v>214</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>60</v>
@@ -3243,28 +3583,28 @@
         <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D2" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="E2" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G2" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="H2">
         <v>869308</v>
       </c>
       <c r="I2" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="J2" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="K2" t="s">
         <v>67</v>
@@ -3278,28 +3618,28 @@
         <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D3" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="E3" t="s">
-        <v>202</v>
+        <v>223</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G3" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="H3">
         <v>869308</v>
       </c>
       <c r="I3" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="J3" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="K3" t="s">
         <v>75</v>
@@ -3313,28 +3653,28 @@
         <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="D4" t="s">
-        <v>204</v>
+        <v>225</v>
       </c>
       <c r="E4" t="s">
-        <v>205</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G4" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="H4">
         <v>12539</v>
       </c>
       <c r="I4" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="J4" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="K4" t="s">
         <v>81</v>
@@ -3348,28 +3688,28 @@
         <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D5" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
       <c r="E5" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G5" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="H5">
         <v>869308</v>
       </c>
       <c r="I5" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="J5" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="K5" t="s">
         <v>85</v>
@@ -3383,28 +3723,28 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D6" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="E6" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G6" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="H6">
         <v>869308</v>
       </c>
       <c r="I6" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="J6" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="K6" t="s">
         <v>92</v>
@@ -3418,34 +3758,69 @@
         <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="D7" t="s">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="E7" t="s">
-        <v>213</v>
+        <v>234</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G7" t="s">
-        <v>214</v>
+        <v>235</v>
       </c>
       <c r="H7">
         <v>115</v>
       </c>
       <c r="I7" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="J7" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="K7" t="s">
         <v>97</v>
       </c>
       <c r="L7" t="s">
         <v>99</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" t="s">
+        <v>216</v>
+      </c>
+      <c r="D8" t="s">
+        <v>237</v>
+      </c>
+      <c r="E8" t="s">
+        <v>238</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G8" t="s">
+        <v>219</v>
+      </c>
+      <c r="H8">
+        <v>869308</v>
+      </c>
+      <c r="I8" t="s">
+        <v>220</v>
+      </c>
+      <c r="J8" t="s">
+        <v>221</v>
+      </c>
+      <c r="K8" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -3456,9 +3831,10 @@
     <hyperlink ref="F5" r:id="rId4"/>
     <hyperlink ref="F6" r:id="rId5"/>
     <hyperlink ref="F7" r:id="rId6"/>
+    <hyperlink ref="F8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: granular number-level approval and rejection with remarks and resubmission support
</commit_message>
<xml_diff>
--- a/shared/CallerID-Database.xlsx
+++ b/shared/CallerID-Database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="272">
   <si>
     <t>packageId</t>
   </si>
@@ -169,6 +169,18 @@
     <t>2026-10-27T09:33:52.890Z</t>
   </si>
   <si>
+    <t>PKG-c70e68ea</t>
+  </si>
+  <si>
+    <t>evening 27</t>
+  </si>
+  <si>
+    <t>2026-10-27T13:38:04.045Z</t>
+  </si>
+  <si>
+    <t>15 Days</t>
+  </si>
+  <si>
     <t>requestId</t>
   </si>
   <si>
@@ -325,7 +337,7 @@
     <t>Exclusive Diwali Offer</t>
   </si>
   <si>
-    <t>pending</t>
+    <t>partially approved</t>
   </si>
   <si>
     <t>FILE-3204d32b</t>
@@ -337,6 +349,24 @@
     <t>Customer Service</t>
   </si>
   <si>
+    <t>Invalid department direct line</t>
+  </si>
+  <si>
+    <t>REQ-c1604260</t>
+  </si>
+  <si>
+    <t>FILE-a5b6ab26</t>
+  </si>
+  <si>
+    <t>2026-10-27T13:39:18.432Z</t>
+  </si>
+  <si>
+    <t>Marketing, Credit Cards, Customer Service</t>
+  </si>
+  <si>
+    <t>unknown no</t>
+  </si>
+  <si>
     <t>numberId</t>
   </si>
   <si>
@@ -352,6 +382,9 @@
     <t>numberType</t>
   </si>
   <si>
+    <t>decidedAt</t>
+  </si>
+  <si>
     <t>NUM-3c3cf48e</t>
   </si>
   <si>
@@ -598,6 +631,9 @@
     <t>+63 939 838 6747</t>
   </si>
   <si>
+    <t>2026-10-27T16:52:02.087Z</t>
+  </si>
+  <si>
     <t>NUM-8f6f703f</t>
   </si>
   <si>
@@ -634,6 +670,54 @@
     <t>+63 919 221 6074</t>
   </si>
   <si>
+    <t>NUM-3b0a9267</t>
+  </si>
+  <si>
+    <t>+639772568619</t>
+  </si>
+  <si>
+    <t>+63 977 256 8619</t>
+  </si>
+  <si>
+    <t>2026-10-27T16:55:49.380Z</t>
+  </si>
+  <si>
+    <t>NUM-593a6dcb</t>
+  </si>
+  <si>
+    <t>+639184082877</t>
+  </si>
+  <si>
+    <t>+63 918 408 2877</t>
+  </si>
+  <si>
+    <t>NUM-b60d5013</t>
+  </si>
+  <si>
+    <t>+639226729359</t>
+  </si>
+  <si>
+    <t>+63 922 672 9359</t>
+  </si>
+  <si>
+    <t>NUM-20cdf77e</t>
+  </si>
+  <si>
+    <t>+639274571153</t>
+  </si>
+  <si>
+    <t>+63 927 457 1153</t>
+  </si>
+  <si>
+    <t>NUM-cd40a9e3</t>
+  </si>
+  <si>
+    <t>+639775773978</t>
+  </si>
+  <si>
+    <t>+63 977 577 3978</t>
+  </si>
+  <si>
     <t>fileId</t>
   </si>
   <si>
@@ -731,6 +815,21 @@
   </si>
   <si>
     <t>storage/logos/FILE-3204d32b.png</t>
+  </si>
+  <si>
+    <t>metro bank.jpeg</t>
+  </si>
+  <si>
+    <t>FILE-a5b6ab26.jpg</t>
+  </si>
+  <si>
+    <t>storage/logos/FILE-a5b6ab26.jpg</t>
+  </si>
+  <si>
+    <t>image/jpeg</t>
+  </si>
+  <si>
+    <t>926d51fb661f44bd9c12e38b452f0a32917ccefc90fe40416b2dc483811323b5</t>
   </si>
 </sst>
 </file>
@@ -1034,6 +1133,45 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>13999</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>17999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="533400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1257,6 +1395,45 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>13999</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>17999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="533400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1598,7 +1775,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="14" customWidth="1"/>
@@ -2012,6 +2189,44 @@
         <v>1</v>
       </c>
     </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14" s="2">
+        <v>15000</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" t="s">
+        <v>54</v>
+      </c>
+      <c r="K14">
+        <v>50000</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -2020,7 +2235,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="14" customWidth="1"/>
@@ -2032,13 +2247,13 @@
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
@@ -2047,63 +2262,63 @@
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I2">
         <v>5</v>
@@ -2118,33 +2333,33 @@
         <v>16800</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I3">
         <v>4</v>
@@ -2159,33 +2374,33 @@
         <v>22400</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I4">
         <v>5</v>
@@ -2200,33 +2415,33 @@
         <v>16800</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I5">
         <v>5</v>
@@ -2241,33 +2456,33 @@
         <v>16800</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I6">
         <v>5</v>
@@ -2284,28 +2499,28 @@
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
         <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G7" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -2320,33 +2535,33 @@
         <v>16800</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
         <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="H8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I8">
         <v>2</v>
@@ -2361,42 +2576,42 @@
         <v>16800</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N8" t="s">
+        <v>103</v>
+      </c>
+      <c r="O8" t="s">
         <v>99</v>
       </c>
-      <c r="O8" t="s">
-        <v>95</v>
-      </c>
       <c r="P8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G9" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H9" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I9">
         <v>5</v>
@@ -2411,13 +2626,60 @@
         <v>16800</v>
       </c>
       <c r="M9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="O9" t="s">
+        <v>106</v>
+      </c>
+      <c r="P9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" t="s">
         <v>69</v>
       </c>
-      <c r="O9" t="s">
-        <v>102</v>
-      </c>
-      <c r="P9" t="s">
-        <v>64</v>
+      <c r="F10" t="s">
+        <v>113</v>
+      </c>
+      <c r="G10" t="s">
+        <v>114</v>
+      </c>
+      <c r="H10" t="s">
+        <v>115</v>
+      </c>
+      <c r="I10">
+        <v>5</v>
+      </c>
+      <c r="J10" s="2">
+        <v>15000</v>
+      </c>
+      <c r="K10" s="2">
+        <v>1800</v>
+      </c>
+      <c r="L10" s="2">
+        <v>16800</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="O10" t="s">
+        <v>106</v>
+      </c>
+      <c r="P10" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2429,44 +2691,45 @@
     <hyperlink ref="M7" r:id="rId5"/>
     <hyperlink ref="M8" r:id="rId6"/>
     <hyperlink ref="M9" r:id="rId7"/>
+    <hyperlink ref="M10" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId8"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="9" width="14" customWidth="1"/>
+    <col min="7" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -2474,1049 +2737,1260 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="F2" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="G2" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="F3" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="G3" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E4" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="F4" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="G4" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F5" t="s">
+        <v>138</v>
+      </c>
+      <c r="G5" t="s">
         <v>126</v>
       </c>
-      <c r="F5" t="s">
-        <v>127</v>
-      </c>
-      <c r="G5" t="s">
-        <v>115</v>
-      </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D6" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E6" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="F6" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="G6" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E7" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="F7" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="G7" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E8" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="F8" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="G8" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I8" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D9" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E9" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="F9" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G9" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E10" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="F10" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="G10" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="B11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F11" t="s">
+        <v>125</v>
+      </c>
+      <c r="G11" t="s">
+        <v>126</v>
+      </c>
+      <c r="H11" t="s">
         <v>77</v>
       </c>
-      <c r="C11" t="s">
-        <v>78</v>
-      </c>
-      <c r="D11" t="s">
-        <v>106</v>
-      </c>
-      <c r="E11" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" t="s">
-        <v>114</v>
-      </c>
-      <c r="G11" t="s">
-        <v>115</v>
-      </c>
-      <c r="H11" t="s">
-        <v>73</v>
-      </c>
       <c r="I11" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" t="s">
+        <v>128</v>
+      </c>
+      <c r="F12" t="s">
+        <v>129</v>
+      </c>
+      <c r="G12" t="s">
+        <v>126</v>
+      </c>
+      <c r="H12" t="s">
         <v>77</v>
       </c>
-      <c r="C12" t="s">
-        <v>78</v>
-      </c>
-      <c r="D12" t="s">
-        <v>106</v>
-      </c>
-      <c r="E12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F12" t="s">
-        <v>118</v>
-      </c>
-      <c r="G12" t="s">
-        <v>115</v>
-      </c>
-      <c r="H12" t="s">
-        <v>73</v>
-      </c>
       <c r="I12" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="B13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" t="s">
+        <v>131</v>
+      </c>
+      <c r="E13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F13" t="s">
+        <v>133</v>
+      </c>
+      <c r="G13" t="s">
+        <v>134</v>
+      </c>
+      <c r="H13" t="s">
         <v>77</v>
       </c>
-      <c r="C13" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" t="s">
-        <v>120</v>
-      </c>
-      <c r="E13" t="s">
-        <v>121</v>
-      </c>
-      <c r="F13" t="s">
-        <v>122</v>
-      </c>
-      <c r="G13" t="s">
-        <v>123</v>
-      </c>
-      <c r="H13" t="s">
-        <v>73</v>
-      </c>
       <c r="I13" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="B14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" t="s">
+        <v>137</v>
+      </c>
+      <c r="F14" t="s">
+        <v>138</v>
+      </c>
+      <c r="G14" t="s">
+        <v>126</v>
+      </c>
+      <c r="H14" t="s">
         <v>77</v>
       </c>
-      <c r="C14" t="s">
-        <v>78</v>
-      </c>
-      <c r="D14" t="s">
-        <v>125</v>
-      </c>
-      <c r="E14" t="s">
-        <v>126</v>
-      </c>
-      <c r="F14" t="s">
-        <v>127</v>
-      </c>
-      <c r="G14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H14" t="s">
-        <v>73</v>
-      </c>
       <c r="I14" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="B15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" t="s">
+        <v>141</v>
+      </c>
+      <c r="F15" t="s">
+        <v>142</v>
+      </c>
+      <c r="G15" t="s">
+        <v>143</v>
+      </c>
+      <c r="H15" t="s">
         <v>77</v>
       </c>
-      <c r="C15" t="s">
-        <v>78</v>
-      </c>
-      <c r="D15" t="s">
-        <v>129</v>
-      </c>
-      <c r="E15" t="s">
-        <v>130</v>
-      </c>
-      <c r="F15" t="s">
-        <v>131</v>
-      </c>
-      <c r="G15" t="s">
-        <v>132</v>
-      </c>
-      <c r="H15" t="s">
-        <v>73</v>
-      </c>
       <c r="I15" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E16" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="F16" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="G16" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H16" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="B17" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D17" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E17" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="F17" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="G17" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H17" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I17" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D18" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E18" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="F18" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="G18" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="H18" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I18" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D19" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E19" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="F19" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="G19" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H19" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I19" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="B20" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C20" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D20" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E20" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="F20" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="G20" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="H20" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I20" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="B21" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D21" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E21" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="F21" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="G21" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H21" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I21" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D22" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E22" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="F22" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="G22" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H22" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I22" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D23" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E23" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="F23" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="G23" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="H23" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I23" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D24" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E24" t="s">
+        <v>137</v>
+      </c>
+      <c r="F24" t="s">
+        <v>138</v>
+      </c>
+      <c r="G24" t="s">
         <v>126</v>
       </c>
-      <c r="F24" t="s">
-        <v>127</v>
-      </c>
-      <c r="G24" t="s">
-        <v>115</v>
-      </c>
       <c r="H24" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I24" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D25" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E25" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="F25" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="G25" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="H25" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I25" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D26" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E26" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="F26" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="G26" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H26" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I26" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D27" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E27" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="F27" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="G27" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H27" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I27" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D28" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E28" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="F28" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="G28" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="H28" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I28" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C29" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D29" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E29" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="F29" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="G29" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H29" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I29" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C30" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D30" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E30" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="F30" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="G30" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="H30" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I30" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="B31" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C31" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E31" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="F31" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="G31" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H31" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I31" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D32" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E32" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="F32" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="G32" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H32" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I32" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="B33" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C33" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D33" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E33" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="F33" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="G33" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H33" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="I33" t="s">
+        <v>109</v>
+      </c>
+      <c r="J33" t="s">
+        <v>68</v>
+      </c>
+      <c r="K33" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>206</v>
+      </c>
+      <c r="B34" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>194</v>
-      </c>
-      <c r="B34" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" t="s">
-        <v>101</v>
-      </c>
       <c r="D34" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E34" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="F34" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="G34" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H34" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="I34" t="s">
+        <v>109</v>
+      </c>
+      <c r="J34" t="s">
+        <v>111</v>
+      </c>
+      <c r="K34" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>209</v>
+      </c>
+      <c r="B35" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>197</v>
-      </c>
-      <c r="B35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C35" t="s">
-        <v>101</v>
-      </c>
       <c r="D35" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E35" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="F35" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="G35" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H35" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="I35" t="s">
+        <v>109</v>
+      </c>
+      <c r="J35" t="s">
+        <v>111</v>
+      </c>
+      <c r="K35" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>212</v>
+      </c>
+      <c r="B36" t="s">
+        <v>104</v>
+      </c>
+      <c r="C36" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>200</v>
-      </c>
-      <c r="B36" t="s">
-        <v>100</v>
-      </c>
-      <c r="C36" t="s">
-        <v>101</v>
-      </c>
       <c r="D36" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E36" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="F36" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="G36" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H36" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="I36" t="s">
+        <v>109</v>
+      </c>
+      <c r="J36" t="s">
+        <v>111</v>
+      </c>
+      <c r="K36" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>215</v>
+      </c>
+      <c r="B37" t="s">
+        <v>104</v>
+      </c>
+      <c r="C37" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>203</v>
-      </c>
-      <c r="B37" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" t="s">
-        <v>101</v>
-      </c>
       <c r="D37" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E37" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="F37" t="s">
+        <v>217</v>
+      </c>
+      <c r="G37" t="s">
+        <v>126</v>
+      </c>
+      <c r="H37" t="s">
+        <v>77</v>
+      </c>
+      <c r="I37" t="s">
+        <v>109</v>
+      </c>
+      <c r="J37" t="s">
+        <v>68</v>
+      </c>
+      <c r="K37" t="s">
         <v>205</v>
       </c>
-      <c r="G37" t="s">
-        <v>115</v>
-      </c>
-      <c r="H37" t="s">
-        <v>103</v>
-      </c>
-      <c r="I37" t="s">
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>218</v>
+      </c>
+      <c r="B38" t="s">
+        <v>112</v>
+      </c>
+      <c r="C38" t="s">
         <v>105</v>
+      </c>
+      <c r="D38" t="s">
+        <v>102</v>
+      </c>
+      <c r="E38" t="s">
+        <v>219</v>
+      </c>
+      <c r="F38" t="s">
+        <v>220</v>
+      </c>
+      <c r="G38" t="s">
+        <v>126</v>
+      </c>
+      <c r="H38" t="s">
+        <v>69</v>
+      </c>
+      <c r="I38" t="s">
+        <v>114</v>
+      </c>
+      <c r="J38" t="s">
+        <v>116</v>
+      </c>
+      <c r="K38" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>222</v>
+      </c>
+      <c r="B39" t="s">
+        <v>112</v>
+      </c>
+      <c r="C39" t="s">
+        <v>105</v>
+      </c>
+      <c r="D39" t="s">
+        <v>136</v>
+      </c>
+      <c r="E39" t="s">
+        <v>223</v>
+      </c>
+      <c r="F39" t="s">
+        <v>224</v>
+      </c>
+      <c r="G39" t="s">
+        <v>126</v>
+      </c>
+      <c r="H39" t="s">
+        <v>69</v>
+      </c>
+      <c r="I39" t="s">
+        <v>114</v>
+      </c>
+      <c r="J39" t="s">
+        <v>116</v>
+      </c>
+      <c r="K39" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>225</v>
+      </c>
+      <c r="B40" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" t="s">
+        <v>110</v>
+      </c>
+      <c r="E40" t="s">
+        <v>226</v>
+      </c>
+      <c r="F40" t="s">
+        <v>227</v>
+      </c>
+      <c r="G40" t="s">
+        <v>126</v>
+      </c>
+      <c r="H40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I40" t="s">
+        <v>114</v>
+      </c>
+      <c r="J40" t="s">
+        <v>116</v>
+      </c>
+      <c r="K40" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>228</v>
+      </c>
+      <c r="B41" t="s">
+        <v>112</v>
+      </c>
+      <c r="C41" t="s">
+        <v>105</v>
+      </c>
+      <c r="D41" t="s">
+        <v>110</v>
+      </c>
+      <c r="E41" t="s">
+        <v>229</v>
+      </c>
+      <c r="F41" t="s">
+        <v>230</v>
+      </c>
+      <c r="G41" t="s">
+        <v>126</v>
+      </c>
+      <c r="H41" t="s">
+        <v>69</v>
+      </c>
+      <c r="I41" t="s">
+        <v>114</v>
+      </c>
+      <c r="J41" t="s">
+        <v>116</v>
+      </c>
+      <c r="K41" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>231</v>
+      </c>
+      <c r="B42" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" t="s">
+        <v>105</v>
+      </c>
+      <c r="D42" t="s">
+        <v>110</v>
+      </c>
+      <c r="E42" t="s">
+        <v>232</v>
+      </c>
+      <c r="F42" t="s">
+        <v>233</v>
+      </c>
+      <c r="G42" t="s">
+        <v>126</v>
+      </c>
+      <c r="H42" t="s">
+        <v>69</v>
+      </c>
+      <c r="I42" t="s">
+        <v>114</v>
+      </c>
+      <c r="J42" t="s">
+        <v>116</v>
+      </c>
+      <c r="K42" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -3527,7 +4001,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -3539,288 +4013,323 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>234</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>208</v>
+        <v>236</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>209</v>
+        <v>237</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>211</v>
+        <v>239</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>240</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>213</v>
+        <v>241</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>214</v>
+        <v>242</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>215</v>
+        <v>243</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" t="s">
         <v>66</v>
       </c>
-      <c r="B2" t="s">
-        <v>62</v>
-      </c>
       <c r="C2" t="s">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="D2" t="s">
-        <v>217</v>
+        <v>245</v>
       </c>
       <c r="E2" t="s">
-        <v>218</v>
+        <v>246</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G2" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="H2">
         <v>869308</v>
       </c>
       <c r="I2" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="J2" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s">
         <v>74</v>
       </c>
-      <c r="B3" t="s">
-        <v>70</v>
-      </c>
       <c r="C3" t="s">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="D3" t="s">
-        <v>222</v>
+        <v>250</v>
       </c>
       <c r="E3" t="s">
-        <v>223</v>
+        <v>251</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="H3">
         <v>869308</v>
       </c>
       <c r="I3" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="J3" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="K3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C4" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="D4" t="s">
-        <v>225</v>
+        <v>253</v>
       </c>
       <c r="E4" t="s">
-        <v>226</v>
+        <v>254</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G4" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="H4">
         <v>12539</v>
       </c>
       <c r="I4" t="s">
-        <v>227</v>
+        <v>255</v>
       </c>
       <c r="J4" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C5" t="s">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>256</v>
       </c>
       <c r="E5" t="s">
-        <v>229</v>
+        <v>257</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="H5">
         <v>869308</v>
       </c>
       <c r="I5" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="J5" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="K5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="D6" t="s">
-        <v>230</v>
+        <v>258</v>
       </c>
       <c r="E6" t="s">
-        <v>231</v>
+        <v>259</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G6" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="H6">
         <v>869308</v>
       </c>
       <c r="I6" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="J6" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="K6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>232</v>
+        <v>260</v>
       </c>
       <c r="D7" t="s">
-        <v>233</v>
+        <v>261</v>
       </c>
       <c r="E7" t="s">
-        <v>234</v>
+        <v>262</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G7" t="s">
-        <v>235</v>
+        <v>263</v>
       </c>
       <c r="H7">
         <v>115</v>
       </c>
       <c r="I7" t="s">
-        <v>236</v>
+        <v>264</v>
       </c>
       <c r="J7" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="K7" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" t="s">
         <v>104</v>
       </c>
-      <c r="B8" t="s">
-        <v>100</v>
-      </c>
       <c r="C8" t="s">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="D8" t="s">
-        <v>237</v>
+        <v>265</v>
       </c>
       <c r="E8" t="s">
-        <v>238</v>
+        <v>266</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G8" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="H8">
         <v>869308</v>
       </c>
       <c r="I8" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="J8" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="K8" t="s">
-        <v>105</v>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C9" t="s">
+        <v>267</v>
+      </c>
+      <c r="D9" t="s">
+        <v>268</v>
+      </c>
+      <c r="E9" t="s">
+        <v>269</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" t="s">
+        <v>270</v>
+      </c>
+      <c r="H9">
+        <v>49961</v>
+      </c>
+      <c r="I9" t="s">
+        <v>271</v>
+      </c>
+      <c r="J9" t="s">
+        <v>249</v>
+      </c>
+      <c r="K9" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -3832,9 +4341,10 @@
     <hyperlink ref="F6" r:id="rId5"/>
     <hyperlink ref="F7" r:id="rId6"/>
     <hyperlink ref="F8" r:id="rId7"/>
+    <hyperlink ref="F9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId8"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>